<commit_message>
Auto update ESO load data
</commit_message>
<xml_diff>
--- a/data/plexos_load_master.xlsx
+++ b/data/plexos_load_master.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA24"/>
+  <dimension ref="A1:AA25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2472,6 +2472,89 @@
       </c>
       <c r="AA24" t="n">
         <v>4916</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B25" t="n">
+        <v>2</v>
+      </c>
+      <c r="C25" t="n">
+        <v>28</v>
+      </c>
+      <c r="D25" t="n">
+        <v>4754</v>
+      </c>
+      <c r="E25" t="n">
+        <v>4516</v>
+      </c>
+      <c r="F25" t="n">
+        <v>4397</v>
+      </c>
+      <c r="G25" t="n">
+        <v>4357</v>
+      </c>
+      <c r="H25" t="n">
+        <v>4342</v>
+      </c>
+      <c r="I25" t="n">
+        <v>4399</v>
+      </c>
+      <c r="J25" t="n">
+        <v>4653</v>
+      </c>
+      <c r="K25" t="n">
+        <v>5108</v>
+      </c>
+      <c r="L25" t="n">
+        <v>5488</v>
+      </c>
+      <c r="M25" t="n">
+        <v>5451</v>
+      </c>
+      <c r="N25" t="n">
+        <v>5338</v>
+      </c>
+      <c r="O25" t="n">
+        <v>5258</v>
+      </c>
+      <c r="P25" t="n">
+        <v>5194</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>5169</v>
+      </c>
+      <c r="R25" t="n">
+        <v>5150</v>
+      </c>
+      <c r="S25" t="n">
+        <v>5205</v>
+      </c>
+      <c r="T25" t="n">
+        <v>5311</v>
+      </c>
+      <c r="U25" t="n">
+        <v>5470</v>
+      </c>
+      <c r="V25" t="n">
+        <v>5651</v>
+      </c>
+      <c r="W25" t="n">
+        <v>5559</v>
+      </c>
+      <c r="X25" t="n">
+        <v>5275</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>5043</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>4895</v>
+      </c>
+      <c r="AA25" t="n">
+        <v>4643</v>
       </c>
     </row>
   </sheetData>

</xml_diff>